<commit_message>
fix: Using asset for timeout when getting messages.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RPA\Jonas\RPA_IAF_Rakel_Hamta_Meddelande_Dispatcher\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\RPA\Claes 2\RPA_IAF_Rakel_Hamta_Meddelande_Dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E4AABB-B3F7-4D4E-8E72-1DE0C5BB6227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12570" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="60">
   <si>
     <t>Name</t>
   </si>
@@ -190,13 +191,25 @@
     <t>Rakel Meddelanden och Bilagor Performer Dispatcher</t>
   </si>
   <si>
-    <t>FALSE</t>
+    <t>OeP_URL_PRD</t>
+  </si>
+  <si>
+    <t>Timeout_GetMessages</t>
+  </si>
+  <si>
+    <t>OeP_GetMessagesTimeout</t>
+  </si>
+  <si>
+    <t>In millisecs</t>
+  </si>
+  <si>
+    <t>TRUE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4">
     <font>
       <sz val="11"/>
@@ -565,7 +578,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z998"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -651,7 +664,14 @@
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9">
+        <v>60000</v>
+      </c>
+    </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1649,7 +1669,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z989"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -1834,7 +1854,7 @@
         <v>36</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>38</v>
@@ -2819,8 +2839,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z1000"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:Z996"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
@@ -2916,8 +2936,25 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" t="s">
+        <v>58</v>
+      </c>
+    </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
@@ -3905,12 +3942,9 @@
     <row r="994" ht="14.25" customHeight="1"/>
     <row r="995" ht="14.25" customHeight="1"/>
     <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>